<commit_message>
add week sum 1220
</commit_message>
<xml_diff>
--- a/_posts/工作簿1.xlsx
+++ b/_posts/工作簿1.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mxm\Documents\Code\blog\_posts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E186644-BCD9-4822-A425-28E59ECDCEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F75621E4-0868-4B15-B1A0-FE58A875357B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10800" yWindow="0" windowWidth="10800" windowHeight="13954" xr2:uid="{5772B7EC-0D34-4D98-8C50-8053F9C4DDDF}"/>
+    <workbookView xWindow="-69" yWindow="-69" windowWidth="16595" windowHeight="12035" xr2:uid="{5772B7EC-0D34-4D98-8C50-8053F9C4DDDF}"/>
   </bookViews>
   <sheets>
-    <sheet name="LeggedRobotCfgPPO" sheetId="3" r:id="rId1"/>
-    <sheet name="LeggedRobotCfg" sheetId="2" r:id="rId2"/>
-    <sheet name="BaseTask" sheetId="1" r:id="rId3"/>
+    <sheet name="LeggedRobot" sheetId="4" r:id="rId1"/>
+    <sheet name="LeggedRobotCfgPPO" sheetId="3" r:id="rId2"/>
+    <sheet name="LeggedRobotCfg" sheetId="2" r:id="rId3"/>
+    <sheet name="BaseTask" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="77">
   <si>
     <t>函数名/代码块</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -356,6 +357,49 @@
     <t>OnPolicyRunner定义了整个训练过程，包含learn, log, save等过程
 PPO为训练模型的一种方法
 ActorCritic应该是强化学习方法</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>`__init__(self, cfg, …)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>初始化类的属性
+设置viewer-camera
+映射reward scale-function</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">`self._parse_cfg(cfg)`:
+self.dt = decimation*dt # 所以env中的dt就是控制器输出的时间间隔，不是仿真环境的时间间隔
+self.max_episode_length = episode_length_s / dt # 也就是离散时间的采样点n
+self.cfg.domain_rand.push_interval: 同上
+所以**env中的时间概念都是离散时间的采样点n，离散时间的周期是仿真周期*decimation**
+`super().__init__()`:
+self.num_envs/num_obs/num_priviledge_obs/num_actions都有cfg中定义而来
+self.obs_buf: shape = (num_envs, num_obs,) 自定义obs维度
+self.rew_buf: shape = (num_envs,) 每个环境都有一个reward value记录
+self.reset_buf: shape = (num_envs, ) 每个环境一个reset flag True/False
+self.episode_length_buf: shape = (num, envs,) 记录当前trial/episode经过的时刻n
+self.time_out_buf: shape = (num_envs, )应该是存放一个最大时间来判断
+self.create_sim(): 在BaseTask中调用，但是在LeggedRobot中定义。
+`self.create_sim()`:
+self.up_axis_idx = 2 # 2 for z, 1 for y, 设置重力方向
+self._create_envs()
+`self._create_envs()`:
+加载assets
+self.dof_names: list of str，从asset文件中获取
+self.num_dofs # len(self.dof_names)，应该 == cfg.num_actions
+self.base_init_state: 加载由cfg中定义的init_state.pos/rot/lin_vel/ang_vel
+定义envs/actors，并且保存handle(引用) -&gt; self.envs / self.actor_handles: list of handle
+self.feet_indices / self.penalised_contact_indices / self.termination_contact_indices: 根据cfg.asset.foot_name等，根据self.gym.find_actor_rigid_body_handle(self.envs[0], self.actor_handles[0], feet_name[i])来获取索引
+`self._init_buffers()`: 从仿真gym中获取各种状态，建立其引用。则当self.gym.acquire/refresh时，对应的tensor就会自动更新，
+self.root_states: shape= (num_envs, 13) # 13=3pos+4rot+3lin_vel+3ang_vel
+self.dof_state: shape=(num_envs * num_actions, 2) # 2 = 位置与速度
+self.dof_pos: shape = (num_envs, num_actions)
+self.dof_vel: shape = (num_envs, num_actions)
+self.base_quat: shape = (num_envs, 4) # root坐标系相对世界坐标系的旋转四元数
+</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -745,6 +789,47 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6B5FDB5-7724-4DBB-942F-4DB53D5A0685}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.0703125" customWidth="1"/>
+    <col min="2" max="2" width="26.2109375" customWidth="1"/>
+    <col min="3" max="3" width="79.5" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="5" width="28.35546875" customWidth="1"/>
+    <col min="6" max="6" width="42.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="42.45" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="409.6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50328ED3-D70A-43B4-9611-5AD33549D9AB}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
@@ -832,7 +917,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73EC9D5E-E984-42F1-9294-81606E8BCB14}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
@@ -980,7 +1065,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C5FA566-A393-4223-98D0-56D6655EFC9C}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>

</xml_diff>